<commit_message>
Resolve case-insensitive dataset paths
</commit_message>
<xml_diff>
--- a/Data/Comparison_Results/manual_review.xlsx
+++ b/Data/Comparison_Results/manual_review.xlsx
@@ -690,10 +690,10 @@
     <t>supertest</t>
   </si>
   <si>
-    <t>App.test_1</t>
-  </si>
-  <si>
-    <t>App.test_2</t>
+    <t>send_message.test_1</t>
+  </si>
+  <si>
+    <t>send_message.test_2</t>
   </si>
   <si>
     <t>api.test_1_1</t>

</xml_diff>

<commit_message>
Remove contact details and document metadata
</commit_message>
<xml_diff>
--- a/Data/Comparison_Results/manual_review.xlsx
+++ b/Data/Comparison_Results/manual_review.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yundong/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053E3452-7C6C-8540-8F66-32042F6DDFD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>